<commit_message>
Data update 2026-09-11 10:11
</commit_message>
<xml_diff>
--- a/Database/Cecafe Monthly.xlsx
+++ b/Database/Cecafe Monthly.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://etgworld.sharepoint.com/sites/SoftsDatabase/Shared Documents/Database/Hardmine/Fundamental/Cecafe Monthly/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_D27E3E97F52CB5635F469446D970799563192C1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBED71B2-8E99-4A86-8F5E-EBEA25D0C1A7}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="11_D27E3E97F52CB5635F469446D970799563192C1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2342290F-F6D6-4F19-A874-6DA1C943B3A0}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8663" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8703" uniqueCount="20">
   <si>
     <t>Year</t>
   </si>
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4330"/>
+  <dimension ref="A1:E4350"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -74038,6 +74038,346 @@
       </c>
       <c r="E4330">
         <v>31.7</v>
+      </c>
+    </row>
+    <row r="4331" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4331">
+        <v>2026</v>
+      </c>
+      <c r="B4331">
+        <v>8</v>
+      </c>
+      <c r="C4331" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4331" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4331">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="4332" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4332">
+        <v>2026</v>
+      </c>
+      <c r="B4332">
+        <v>8</v>
+      </c>
+      <c r="C4332" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4332" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4332">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="4333" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4333">
+        <v>2026</v>
+      </c>
+      <c r="B4333">
+        <v>8</v>
+      </c>
+      <c r="C4333" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4333" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4333">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="4334" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4334">
+        <v>2026</v>
+      </c>
+      <c r="B4334">
+        <v>8</v>
+      </c>
+      <c r="C4334" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4334" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4334">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4335" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4335">
+        <v>2026</v>
+      </c>
+      <c r="B4335">
+        <v>8</v>
+      </c>
+      <c r="C4335" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4335" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4335">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="4336" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4336">
+        <v>2026</v>
+      </c>
+      <c r="B4336">
+        <v>8</v>
+      </c>
+      <c r="C4336" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4336" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4336">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4337" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4337">
+        <v>2026</v>
+      </c>
+      <c r="B4337">
+        <v>8</v>
+      </c>
+      <c r="C4337" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4337" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4337">
+        <v>2867</v>
+      </c>
+    </row>
+    <row r="4338" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4338">
+        <v>2026</v>
+      </c>
+      <c r="B4338">
+        <v>8</v>
+      </c>
+      <c r="C4338" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4338" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4338">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4339" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4339">
+        <v>2026</v>
+      </c>
+      <c r="B4339">
+        <v>8</v>
+      </c>
+      <c r="C4339" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4339" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4339">
+        <v>41.2</v>
+      </c>
+    </row>
+    <row r="4340" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4340">
+        <v>2026</v>
+      </c>
+      <c r="B4340">
+        <v>8</v>
+      </c>
+      <c r="C4340" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4340" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4340">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="4341" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4341">
+        <v>2026</v>
+      </c>
+      <c r="B4341">
+        <v>8</v>
+      </c>
+      <c r="C4341" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4341" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4341">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4342" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4342">
+        <v>2026</v>
+      </c>
+      <c r="B4342">
+        <v>8</v>
+      </c>
+      <c r="C4342" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4342" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4342">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4343" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4343">
+        <v>2026</v>
+      </c>
+      <c r="B4343">
+        <v>8</v>
+      </c>
+      <c r="C4343" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4343" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4343">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4344" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4344">
+        <v>2026</v>
+      </c>
+      <c r="B4344">
+        <v>8</v>
+      </c>
+      <c r="C4344" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4344" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4344">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4345" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4345">
+        <v>2026</v>
+      </c>
+      <c r="B4345">
+        <v>8</v>
+      </c>
+      <c r="C4345" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4345" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4345">
+        <v>52.5</v>
+      </c>
+    </row>
+    <row r="4346" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4346">
+        <v>2026</v>
+      </c>
+      <c r="B4346">
+        <v>8</v>
+      </c>
+      <c r="C4346" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4346" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4346">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4347" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4347">
+        <v>2026</v>
+      </c>
+      <c r="B4347">
+        <v>8</v>
+      </c>
+      <c r="C4347" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4347" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4347">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="4348" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4348">
+        <v>2026</v>
+      </c>
+      <c r="B4348">
+        <v>8</v>
+      </c>
+      <c r="C4348" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4348" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4348">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4349" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4349">
+        <v>2026</v>
+      </c>
+      <c r="B4349">
+        <v>8</v>
+      </c>
+      <c r="C4349" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4349" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4349">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="4350" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4350">
+        <v>2026</v>
+      </c>
+      <c r="B4350">
+        <v>8</v>
+      </c>
+      <c r="C4350" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4350" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4350">
+        <v>25.3</v>
       </c>
     </row>
   </sheetData>
@@ -74046,12 +74386,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bb8a688-9fce-46e7-b438-b3767c5bce2d" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -74244,20 +74586,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3bb8a688-9fce-46e7-b438-b3767c5bce2d" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8AF0BEB-E956-46BE-8CC2-336EC21D779F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F67B1F73-1EE6-47CB-9CA3-2D73748DC068}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3bb8a688-9fce-46e7-b438-b3767c5bce2d"/>
+    <ds:schemaRef ds:uri="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -74282,12 +74625,15 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F67B1F73-1EE6-47CB-9CA3-2D73748DC068}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8AF0BEB-E956-46BE-8CC2-336EC21D779F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3bb8a688-9fce-46e7-b438-b3767c5bce2d"/>
-    <ds:schemaRef ds:uri="4315a1d7-5b2b-4aec-b3c1-bed157ad3cff"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9324bd15-b7b3-4e59-b23e-9f53050507bb}" enabled="0" method="" siteId="{9324bd15-b7b3-4e59-b23e-9f53050507bb}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>